<commit_message>
docs: atualizar fichamento para a lista final de 30 artigos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018mG9JxEpndiaMffzRmJL2M
</commit_message>
<xml_diff>
--- a/TCC/Fichamento_TCC_facetas_diretas.xlsx
+++ b/TCC/Fichamento_TCC_facetas_diretas.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Progresso por tópico" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Artigos!$A$4:$L$35</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Artigos!$A$4:$L$34</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,9 +24,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="175">
-  <si>
-    <t xml:space="preserve">TCC – Faceta direta em resina composta: fichamento dos 31 artigos</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="165">
+  <si>
+    <t xml:space="preserve">TCC – Faceta direta em resina composta: fichamento dos 30 artigos</t>
   </si>
   <si>
     <t xml:space="preserve">Como usar: as colunas J, K e L (em amarelo) são para você marcar 'Sim' conforme avança. Dentro de cada tópico, os artigos estão em ordem de ano, que é a ordem em que entram na Revisão de Literatura. A coluna 'Atenção' (em vermelho) aponta o que precisa ser resolvido.</t>
@@ -182,6 +182,24 @@
     <t xml:space="preserve">4.2 Resinas compostas: propriedades e estabilidade</t>
   </si>
   <si>
+    <t xml:space="preserve">Irgang et al. (2020)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estudo clínico retrospectivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Journal of Research in Dentistry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avaliação de 74 facetas diretas em 28 pacientes (6 meses a 10 anos em boca), resina microparticulada x universal, critérios FDI e USPHS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">77% de sobrevida; resina microparticulada teve melhor brilho, menos manchamento, melhor cor e adaptação marginal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Substitui o Manauta. Artigo em inglês.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fernandes et al. (2022)</t>
   </si>
   <si>
@@ -197,24 +215,6 @@
     <t xml:space="preserve">Técnica imediata e resina Z350 XT apresentaram maior dureza.</t>
   </si>
   <si>
-    <t xml:space="preserve">Abdulateef e Çobanoğlu (2022)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ensaio clínico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Journal of Baghdad College of Dentistry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estabilidade de cor de facetas diretas com 4 resinas diferentes após 12 meses (25 pacientes, 57 facetas).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sem diferença significativa entre as resinas; todas com alteração de cor clinicamente aceitável em 1 ano.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PDF incompleto (faltam resultados e discussão): baixe o artigo completo. Artigo em inglês.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tozo-Burgos, Escalante-Otárola e Sánchez-Tito (2025)</t>
   </si>
   <si>
@@ -368,27 +368,6 @@
     <t xml:space="preserve">Confirme o sobrenome do 1º autor (o PDF mostra 'Venkat Ramana Reddy' e 'Vookanti'). Artigo em inglês.</t>
   </si>
   <si>
-    <t xml:space="preserve">Manauta (s.d.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s.d.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Material de fabricante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Polydentia (catálogo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caso de 4 facetas diretas com a matriz Unica anterior (paciente de 52 anos).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conclui destacando a matriz do fabricante.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NÃO é artigo científico (material de marketing, sem data). Recomendo substituir.</t>
-  </si>
-  <si>
     <t xml:space="preserve">4.5 Facetas diretas e o periodonto</t>
   </si>
   <si>
@@ -467,9 +446,6 @@
     <t xml:space="preserve">2009</t>
   </si>
   <si>
-    <t xml:space="preserve">Estudo clínico retrospectivo</t>
-  </si>
-  <si>
     <t xml:space="preserve">British Dental Journal</t>
   </si>
   <si>
@@ -491,22 +467,16 @@
     <t xml:space="preserve">As facetas anteriores são de CERÂMICA: use só para comparação.</t>
   </si>
   <si>
-    <t xml:space="preserve">Josic et al. (2023)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revisão sistemática e meta-análise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dental Materials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Longevidade de restaurações diretas x indiretas em resina em dentes POSTERIORES.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Longevidade semelhante; qualidade de evidência muito baixa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trata de dentes posteriores, não de facetas. Use só como apoio ou substitua. Artigo em inglês.</t>
+    <t xml:space="preserve">Teixeira et al. (2022)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longevidade de facetas diretas (resina) x indiretas (porcelana) em dentes anteriores; só estudos clínicos do PubMed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indiretas tiveram sobrevida um pouco maior e mais estabilidade de cor; diretas são mais fáceis de ajustar forma e cor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Substitui o Josic. Discorda de Galvão et al. (2025): ótimo para a Discussão.</t>
   </si>
   <si>
     <t xml:space="preserve">Galvão et al. (2025)</t>
@@ -1265,7 +1235,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1564,7 +1534,7 @@
         <v>52</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>53</v>
@@ -1578,7 +1548,9 @@
       <c r="H12" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="I12" s="9"/>
+      <c r="I12" s="9" t="s">
+        <v>57</v>
+      </c>
       <c r="J12" s="10"/>
       <c r="K12" s="10"/>
       <c r="L12" s="10"/>
@@ -1591,26 +1563,24 @@
         <v>51</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>28</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="I13" s="9" t="s">
         <v>62</v>
       </c>
+      <c r="I13" s="9"/>
       <c r="J13" s="10"/>
       <c r="K13" s="10"/>
       <c r="L13" s="10"/>
@@ -1629,7 +1599,7 @@
         <v>46</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>64</v>
@@ -1954,65 +1924,63 @@
       <c r="L24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="n">
+      <c r="A25" s="17" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="16" t="s">
-        <v>84</v>
+      <c r="B25" s="18" t="s">
+        <v>114</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>115</v>
+        <v>22</v>
       </c>
       <c r="E25" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F25" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="G25" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="H25" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="H25" s="8" t="s">
-        <v>119</v>
-      </c>
       <c r="I25" s="9" t="s">
-        <v>120</v>
+        <v>26</v>
       </c>
       <c r="J25" s="10"/>
       <c r="K25" s="10"/>
       <c r="L25" s="10"/>
     </row>
-    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="n">
         <v>22</v>
       </c>
       <c r="B26" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="H26" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="C26" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="H26" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="I26" s="9" t="s">
-        <v>26</v>
-      </c>
+      <c r="I26" s="9"/>
       <c r="J26" s="10"/>
       <c r="K26" s="10"/>
       <c r="L26" s="10"/>
@@ -2022,70 +1990,70 @@
         <v>23</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>34</v>
+        <v>123</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I27" s="9"/>
       <c r="J27" s="10"/>
       <c r="K27" s="10"/>
       <c r="L27" s="10"/>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="n">
+    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="18" t="s">
-        <v>121</v>
+      <c r="B28" s="20" t="s">
+        <v>126</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="E28" s="8" t="s">
         <v>70</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>130</v>
+        <v>92</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I28" s="9"/>
       <c r="J28" s="10"/>
       <c r="K28" s="10"/>
       <c r="L28" s="10"/>
     </row>
-    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="n">
         <v>25</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>22</v>
@@ -2094,15 +2062,17 @@
         <v>70</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>92</v>
+        <v>34</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="I29" s="9"/>
+        <v>132</v>
+      </c>
+      <c r="I29" s="9" t="s">
+        <v>133</v>
+      </c>
       <c r="J29" s="10"/>
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>
@@ -2112,90 +2082,90 @@
         <v>26</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="I30" s="9" t="s">
-        <v>140</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="I30" s="9"/>
       <c r="J30" s="10"/>
       <c r="K30" s="10"/>
       <c r="L30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="19" t="n">
+      <c r="A31" s="21" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="20" t="s">
-        <v>133</v>
+      <c r="B31" s="22" t="s">
+        <v>137</v>
       </c>
       <c r="C31" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="G31" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="D31" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G31" s="8" t="s">
+      <c r="H31" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="H31" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="I31" s="9"/>
+      <c r="I31" s="9" t="s">
+        <v>50</v>
+      </c>
       <c r="J31" s="10"/>
       <c r="K31" s="10"/>
       <c r="L31" s="10"/>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="n">
         <v>28</v>
       </c>
       <c r="B32" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="G32" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="H32" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="I32" s="9" t="s">
         <v>146</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="H32" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="I32" s="9" t="s">
-        <v>50</v>
       </c>
       <c r="J32" s="10"/>
       <c r="K32" s="10"/>
@@ -2206,104 +2176,72 @@
         <v>29</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>28</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>70</v>
+        <v>33</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>123</v>
+        <v>34</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="J33" s="10"/>
       <c r="K33" s="10"/>
       <c r="L33" s="10"/>
     </row>
-    <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="21" t="n">
         <v>30</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="C34" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="H34" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="D34" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E34" s="8" t="s">
+      <c r="I34" s="9" t="s">
         <v>156</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="G34" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="H34" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="I34" s="9" t="s">
-        <v>160</v>
       </c>
       <c r="J34" s="10"/>
       <c r="K34" s="10"/>
       <c r="L34" s="10"/>
     </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="21" t="n">
-        <v>31</v>
-      </c>
-      <c r="B35" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="H35" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="I35" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:L35"/>
+  <autoFilter ref="A4:L34"/>
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:L35" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:L34" type="list">
       <formula1>"Sim,Não"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2333,27 +2271,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2361,19 +2299,19 @@
         <v>14</v>
       </c>
       <c r="B4" s="25" t="n">
-        <f aca="false">COUNTIF(Artigos!$B$5:$B$35,A4)</f>
+        <f aca="false">COUNTIF(Artigos!$B$5:$B$34,A4)</f>
         <v>7</v>
       </c>
       <c r="C4" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A4,Artigos!$J$5:$J$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A4,Artigos!$J$5:$J$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="D4" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A4,Artigos!$K$5:$K$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A4,Artigos!$K$5:$K$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="E4" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A4,Artigos!$L$5:$L$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A4,Artigos!$L$5:$L$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="F4" s="26" t="n">
@@ -2386,19 +2324,19 @@
         <v>51</v>
       </c>
       <c r="B5" s="25" t="n">
-        <f aca="false">COUNTIF(Artigos!$B$5:$B$35,A5)</f>
+        <f aca="false">COUNTIF(Artigos!$B$5:$B$34,A5)</f>
         <v>3</v>
       </c>
       <c r="C5" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A5,Artigos!$J$5:$J$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A5,Artigos!$J$5:$J$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="D5" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A5,Artigos!$K$5:$K$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A5,Artigos!$K$5:$K$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="E5" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A5,Artigos!$L$5:$L$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A5,Artigos!$L$5:$L$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="F5" s="26" t="n">
@@ -2411,19 +2349,19 @@
         <v>67</v>
       </c>
       <c r="B6" s="25" t="n">
-        <f aca="false">COUNTIF(Artigos!$B$5:$B$35,A6)</f>
+        <f aca="false">COUNTIF(Artigos!$B$5:$B$34,A6)</f>
         <v>4</v>
       </c>
       <c r="C6" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A6,Artigos!$J$5:$J$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A6,Artigos!$J$5:$J$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="D6" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A6,Artigos!$K$5:$K$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A6,Artigos!$K$5:$K$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="E6" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A6,Artigos!$L$5:$L$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A6,Artigos!$L$5:$L$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="F6" s="26" t="n">
@@ -2436,19 +2374,19 @@
         <v>84</v>
       </c>
       <c r="B7" s="25" t="n">
-        <f aca="false">COUNTIF(Artigos!$B$5:$B$35,A7)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF(Artigos!$B$5:$B$34,A7)</f>
+        <v>6</v>
       </c>
       <c r="C7" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A7,Artigos!$J$5:$J$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A7,Artigos!$J$5:$J$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="D7" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A7,Artigos!$K$5:$K$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A7,Artigos!$K$5:$K$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="E7" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A7,Artigos!$L$5:$L$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A7,Artigos!$L$5:$L$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="F7" s="26" t="n">
@@ -2458,22 +2396,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="30" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="B8" s="25" t="n">
-        <f aca="false">COUNTIF(Artigos!$B$5:$B$35,A8)</f>
+        <f aca="false">COUNTIF(Artigos!$B$5:$B$34,A8)</f>
         <v>3</v>
       </c>
       <c r="C8" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A8,Artigos!$J$5:$J$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A8,Artigos!$J$5:$J$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="D8" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A8,Artigos!$K$5:$K$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A8,Artigos!$K$5:$K$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="E8" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A8,Artigos!$L$5:$L$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A8,Artigos!$L$5:$L$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="F8" s="26" t="n">
@@ -2483,22 +2421,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B9" s="25" t="n">
-        <f aca="false">COUNTIF(Artigos!$B$5:$B$35,A9)</f>
+        <f aca="false">COUNTIF(Artigos!$B$5:$B$34,A9)</f>
         <v>3</v>
       </c>
       <c r="C9" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A9,Artigos!$J$5:$J$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A9,Artigos!$J$5:$J$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="D9" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A9,Artigos!$K$5:$K$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A9,Artigos!$K$5:$K$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="E9" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A9,Artigos!$L$5:$L$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A9,Artigos!$L$5:$L$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="F9" s="26" t="n">
@@ -2508,22 +2446,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B10" s="25" t="n">
-        <f aca="false">COUNTIF(Artigos!$B$5:$B$35,A10)</f>
+        <f aca="false">COUNTIF(Artigos!$B$5:$B$34,A10)</f>
         <v>4</v>
       </c>
       <c r="C10" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A10,Artigos!$J$5:$J$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A10,Artigos!$J$5:$J$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="D10" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A10,Artigos!$K$5:$K$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A10,Artigos!$K$5:$K$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="E10" s="25" t="n">
-        <f aca="false">COUNTIFS(Artigos!$B$5:$B$35,A10,Artigos!$L$5:$L$35,"Sim")</f>
+        <f aca="false">COUNTIFS(Artigos!$B$5:$B$34,A10,Artigos!$L$5:$L$34,"Sim")</f>
         <v>0</v>
       </c>
       <c r="F10" s="26" t="n">
@@ -2533,11 +2471,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="33" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="B11" s="34" t="n">
         <f aca="false">SUM(B4:B10)</f>
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="34" t="n">
         <f aca="false">SUM(C4:C10)</f>

</xml_diff>

<commit_message>
docs: ordenar alfabeticamente artigos do mesmo ano no fichamento
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018mG9JxEpndiaMffzRmJL2M
</commit_message>
<xml_diff>
--- a/TCC/Fichamento_TCC_facetas_diretas.xlsx
+++ b/TCC/Fichamento_TCC_facetas_diretas.xlsx
@@ -455,6 +455,18 @@
     <t xml:space="preserve">Melhora estética igual; resina preferida por conservar dente, ser mais rápida e mais barata de reparar.</t>
   </si>
   <si>
+    <t xml:space="preserve">Teixeira et al. (2022)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longevidade de facetas diretas (resina) x indiretas (porcelana) em dentes anteriores; só estudos clínicos do PubMed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indiretas tiveram sobrevida um pouco maior e mais estabilidade de cor; diretas são mais fáceis de ajustar forma e cor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Substitui o Josic. Discorda de Galvão et al. (2025): ótimo para a Discussão.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vaz, Lopes e Toledo Neta (2022)</t>
   </si>
   <si>
@@ -465,18 +477,6 @@
   </si>
   <si>
     <t xml:space="preserve">As facetas anteriores são de CERÂMICA: use só para comparação.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teixeira et al. (2022)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Longevidade de facetas diretas (resina) x indiretas (porcelana) em dentes anteriores; só estudos clínicos do PubMed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indiretas tiveram sobrevida um pouco maior e mais estabilidade de cor; diretas são mais fáceis de ajustar forma e cor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Substitui o Josic. Discorda de Galvão et al. (2025): ótimo para a Discussão.</t>
   </si>
   <si>
     <t xml:space="preserve">Galvão et al. (2025)</t>
@@ -2153,10 +2153,10 @@
         <v>28</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>70</v>
+        <v>33</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="G32" s="8" t="s">
         <v>144</v>
@@ -2185,10 +2185,10 @@
         <v>28</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="G33" s="8" t="s">
         <v>148</v>

</xml_diff>